<commit_message>
Update template usage notes
</commit_message>
<xml_diff>
--- a/FHIR_Testdatengenerator_Vorlage.xlsx
+++ b/FHIR_Testdatengenerator_Vorlage.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" mc:Ignorable="v2">
   <authors>
     <author>tc={53456EDE-EA0E-4F81-8513-8E014A5CAB3D}</author>
   </authors>
@@ -46,10 +46,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Ist Beginn und Enddatum gewünscht?</t>
+          <t xml:space="preserve">Dokumentationszeitpunkt: Zeitpunkt der Diagnosedokumentation. Ein Zeitraum wird hier nicht abgebildet.</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -79,7 +76,7 @@
 </file>
 
 <file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" mc:Ignorable="v2">
   <authors>
     <author>tc={F6F97A4E-3155-436D-952D-08248DE74CD2}</author>
   </authors>
@@ -92,10 +89,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
-    Keine Ahnung, wie die kodiert werden...</t>
+          <t xml:space="preserve">LOINC-Code der klinischen Messung. Wenn kein passender Code vorhanden ist, Bezeichner als Text pflegen und LOINC leer lassen.</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -125,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1984" uniqueCount="1130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2099" uniqueCount="1245">
   <si>
     <t xml:space="preserve">Patient-ID</t>
   </si>
@@ -3515,6 +3509,351 @@
   </si>
   <si>
     <t xml:space="preserve">VALIDATE_STRICT = TRUE</t>
+  </si>
+  <si>
+    <t>Patient-ID ist das Pseudonym im Testdatensatz und wird als FHIR Patient.identifier/id verwendet.</t>
+  </si>
+  <si>
+    <t>Nur Patient-IDs, die in diesem Tabellenblatt vorkommen, werden in den übrigen Tabellenblättern verarbeitet.</t>
+  </si>
+  <si>
+    <t>Eine Zeile erzeugt nur dann eine Patient-Ressource, wenn außer Patient-ID mindestens ein weiterer fachlicher Wert gefüllt ist.</t>
+  </si>
+  <si>
+    <t>Komplett leere Zeilen werden in allen Tabellenblättern ignoriert.</t>
+  </si>
+  <si>
+    <t>Fehlende Werte wirklich leer lassen; keine Platzhalter wie -, / oder n/a eintragen.</t>
+  </si>
+  <si>
+    <t>Wenn ein FHIR-Pflichtfeld nicht anders gefüllt werden kann, setzt der Generator soweit möglich Data Absent Reason unknown.</t>
+  </si>
+  <si>
+    <t>Name und Vorname sind Spezialfälle: leerer Vorname/Nachname wird als DUMMY_NAME bzw. DUMMY_SURNAME ausgegeben.</t>
+  </si>
+  <si>
+    <t>Vorname: offizieller Vorname; leer wird zu DUMMY_NAME.</t>
+  </si>
+  <si>
+    <t>Nachname: offizieller Nachname; leer wird zu DUMMY_SURNAME.</t>
+  </si>
+  <si>
+    <t>Anschrift: Freitext mit Straße, Hausnummer, PLZ und Ort; leer wird als unbekannt gekennzeichnet.</t>
+  </si>
+  <si>
+    <t>Geburtsdatum: bevorzugt TT.MM.JJJJ; Jahresangaben wie JJJJ werden weiterhin akzeptiert.</t>
+  </si>
+  <si>
+    <t>Geschlecht: optional; erkannt werden männlich/weiblich/divers/unbekannt sowie m/w/d/x.</t>
+  </si>
+  <si>
+    <t>Krankenkasse: Institutionskennzeichen oder Freitext; leer wird nicht ausgegeben.</t>
+  </si>
+  <si>
+    <t>Einwilligung: ja/nein-Werte werden nur verarbeitet, wenn Datum Einwilligung gefüllt ist.</t>
+  </si>
+  <si>
+    <t>Datum Einwilligung: Datum, ab dem die Consent-Angaben gelten.</t>
+  </si>
+  <si>
+    <t>PDAT Einwilligung: Patientendaten erheben, speichern und nutzen (prospektiv): ja/nein.</t>
+  </si>
+  <si>
+    <t>KKDAT retro Einwilligung: Krankenkassendaten retrospektiv übertragen, speichern und nutzen: ja/nein.</t>
+  </si>
+  <si>
+    <t>KKDAT Einwilligung: Krankenkassendaten prospektiv übertragen, speichern und nutzen: ja/nein.</t>
+  </si>
+  <si>
+    <t>BIOMAT Einwilligung: Biomaterialien erheben, lagern und nutzen: ja/nein.</t>
+  </si>
+  <si>
+    <t>BIOMAT Zusatz Einwilligung: Zusatzentnahme von Biomaterialien: ja/nein.</t>
+  </si>
+  <si>
+    <t>Die Beispieldaten müssen fachlich nicht plausibel sein; sie zeigen vor allem die unterstützte Struktur.</t>
+  </si>
+  <si>
+    <t>Im Code gesetzte FHIR-Profile für dieses Tabellenblatt:</t>
+  </si>
+  <si>
+    <t>Patient-ID muss in Person vorkommen; leere Patient-ID übernimmt die Patient-ID der vorherigen Zeile.</t>
+  </si>
+  <si>
+    <t>Fall-Nr identifiziert den Einrichtungskontakt pro Patient und wird in Ressourcen anderer Tabellen referenziert.</t>
+  </si>
+  <si>
+    <t>Eine neue Fall-Nr erzeugt einen Encounter Level 1. Fachabteilung erzeugt Level 2, Station/Zimmer/Bett erzeugen Level 3 und Locations.</t>
+  </si>
+  <si>
+    <t>Ohne Fall-Nr kann kein Encounter Level 1 erzeugt werden; Einrichtungskontaktklasse darf dann nicht gefüllt sein.</t>
+  </si>
+  <si>
+    <t>Weitere Ressourcen mit derselben Patient-ID und Fall-Nr verweisen auf den erzeugten Encounter.</t>
+  </si>
+  <si>
+    <t>Start: Beginn des Kontakts als Datum oder Zeitpunkt, bevorzugt TT.MM.JJJJ HH:MM:SS.</t>
+  </si>
+  <si>
+    <t>Ende: Ende des Kontakts als Datum oder Zeitpunkt; leer bedeutet in-progress.</t>
+  </si>
+  <si>
+    <t>Regeln für Encounter und Locations:</t>
+  </si>
+  <si>
+    <t>Nur Zeilen zu Patient-IDs aus Person werden verarbeitet.</t>
+  </si>
+  <si>
+    <t>Zeilen ohne fachliche Angaben werden ignoriert.</t>
+  </si>
+  <si>
+    <t>Die Kombination aus Patient-ID und Fall-Nr sollte eindeutig sein.</t>
+  </si>
+  <si>
+    <t>Fall-Nr ist die zentrale Referenz für Diagnose, Prozedur, Labor, Medikation und Dokumente.</t>
+  </si>
+  <si>
+    <t>Empfehlung: Fall-Nr pro Patient einfach hochzählen.</t>
+  </si>
+  <si>
+    <t>Start setzt Encounter.period.start.</t>
+  </si>
+  <si>
+    <t>Ende setzt Encounter.period.end; bei leerem Ende bleibt period.end weg und status wird in-progress.</t>
+  </si>
+  <si>
+    <t>Einrichtungskontaktklasse: Wert aus der Auswahlliste, z. B. stationaer oder ambulant.</t>
+  </si>
+  <si>
+    <t>Patient-ID muss in Person vorkommen; leere Patient-ID übernimmt die Patient-ID der vorherigen Zeile.</t>
+  </si>
+  <si>
+    <t>Fall-Nr ist optional und verweist auf den Encounter aus Fall.</t>
+  </si>
+  <si>
+    <t>Wenn Fall-Nr gefüllt ist, wird Observation.encounter gesetzt.</t>
+  </si>
+  <si>
+    <t>Wenn Fall-Nr leer ist, wird keine Encounter-Referenz gesetzt.</t>
+  </si>
+  <si>
+    <t>Ohne Fall-Nr kann eine spätere Zuordnung nur über Patient-ID und Zeitstempel erfolgen.</t>
+  </si>
+  <si>
+    <t>LOINC: Code des Laborparameters.</t>
+  </si>
+  <si>
+    <t>Parameter: Freitextbezeichnung des Laborparameters.</t>
+  </si>
+  <si>
+    <t>Messwert: numerischer Wert.</t>
+  </si>
+  <si>
+    <t>Einheit: UCUM-Einheit.</t>
+  </si>
+  <si>
+    <t>Zeitstempel (Abnahme): Zeitpunkt der Probenentnahme bzw. Messung, bevorzugt TT.MM.JJJJ HH:MM:SS.</t>
+  </si>
+  <si>
+    <t>Beispiel: zwei Laborwerte pro Fall.</t>
+  </si>
+  <si>
+    <t>Patient-ID muss in Person vorkommen; leere Patient-ID übernimmt die Patient-ID der vorherigen Zeile.</t>
+  </si>
+  <si>
+    <t>Zeilen ohne gültige Patient-ID werden ignoriert.</t>
+  </si>
+  <si>
+    <t>Fall-Nr ist optional und verweist auf den Encounter aus Fall.</t>
+  </si>
+  <si>
+    <t>Wenn Fall-Nr gefüllt ist, wird Condition.encounter gesetzt.</t>
+  </si>
+  <si>
+    <t>Wenn Fall-Nr leer ist, wird keine Encounter-Referenz gesetzt.</t>
+  </si>
+  <si>
+    <t>Ohne Fall-Nr kann eine spätere Zuordnung nur über Patient-ID und Dokumentationszeitpunkt erfolgen.</t>
+  </si>
+  <si>
+    <t>Bezeichner: Freitextbeschreibung der Diagnose.</t>
+  </si>
+  <si>
+    <t>ICD: vollständiger ICD-10-GM-Code.</t>
+  </si>
+  <si>
+    <t>Dokumentationszeitpunkt: Zeitpunkt der Dokumentation, bevorzugt TT.MM.JJJJ HH:MM:SS.</t>
+  </si>
+  <si>
+    <t>Typ: Diagnosentyp aus der Auswahlliste.</t>
+  </si>
+  <si>
+    <t>Beispiel: erster Fall mit Haupt- und Nebendiagnose, zweiter Fall nur mit Hauptdiagnose.</t>
+  </si>
+  <si>
+    <t>Patient-ID muss in Person vorkommen; leere Patient-ID übernimmt die Patient-ID der vorherigen Zeile.</t>
+  </si>
+  <si>
+    <t>Zeilen ohne gültige Patient-ID werden ignoriert.</t>
+  </si>
+  <si>
+    <t>Fall-Nr ist optional und verweist auf den Encounter aus Fall.</t>
+  </si>
+  <si>
+    <t>Wenn Fall-Nr gefüllt ist, wird Procedure.encounter gesetzt.</t>
+  </si>
+  <si>
+    <t>Wenn Fall-Nr leer ist, wird keine Encounter-Referenz gesetzt.</t>
+  </si>
+  <si>
+    <t>Ohne Fall-Nr kann eine spätere Zuordnung nur über Patient-ID und Dokumentationszeitpunkt erfolgen.</t>
+  </si>
+  <si>
+    <t>Prozedurentext: Freitextbeschreibung der Prozedur.</t>
+  </si>
+  <si>
+    <t>Prozedurencode: OPS-Code der Prozedur.</t>
+  </si>
+  <si>
+    <t>Dokumentationszeitpunkt: Zeitpunkt der Dokumentation bzw. Durchführung, bevorzugt TT.MM.JJJJ HH:MM:SS.</t>
+  </si>
+  <si>
+    <t>Beispiel: zwei Prozeduren pro Fall.</t>
+  </si>
+  <si>
+    <t>Patient-ID muss in Person vorkommen; leere Patient-ID übernimmt die Patient-ID der vorherigen Zeile.</t>
+  </si>
+  <si>
+    <t>Zeilen ohne gültige Patient-ID werden ignoriert.</t>
+  </si>
+  <si>
+    <t>Fall-Nr ist optional und verweist auf den Encounter aus Fall.</t>
+  </si>
+  <si>
+    <t>Wenn Fall-Nr gefüllt ist, wird die Encounter-Referenz gesetzt.</t>
+  </si>
+  <si>
+    <t>Wenn Fall-Nr leer ist, wird keine Encounter-Referenz gesetzt.</t>
+  </si>
+  <si>
+    <t>Ohne Fall-Nr kann eine spätere Zuordnung nur über Patient-ID und Zeitstempel erfolgen.</t>
+  </si>
+  <si>
+    <t>Zeitstempel: Zeitpunkt der Verordnung oder Gabe, bevorzugt TT.MM.JJJJ HH:MM:SS.</t>
+  </si>
+  <si>
+    <t>Medikationstyp: erzeugt je nach Auswahlliste MedicationRequest oder MedicationAdministration.</t>
+  </si>
+  <si>
+    <t>Medikationsplanart: Wert aus der Auswahlliste.</t>
+  </si>
+  <si>
+    <t>Wirksubstanz aus Präparat/Handelsname: Freitext der Medikation.</t>
+  </si>
+  <si>
+    <t>ATC Code und/oder PZN Code der Medikation; ATC wird für die Medication-ID bevorzugt.</t>
+  </si>
+  <si>
+    <t>PZN wird 8-stellig mit führenden Nullen aufgefüllt.</t>
+  </si>
+  <si>
+    <t>ASK: Code des Wirkstoffs; leer wird als unknown gekennzeichnet.</t>
+  </si>
+  <si>
+    <t>FHIR_UserSelected: enthält ATC oder PZN, wenn der jeweilige Code als userSelected markiert werden soll.</t>
+  </si>
+  <si>
+    <t>Darreichungsform: Wert aus der Auswahlliste.</t>
+  </si>
+  <si>
+    <t>Therapiestart: Beginn des Therapiezeitraums.</t>
+  </si>
+  <si>
+    <t>Therapieende: Ende des Therapiezeitraums; leer oder gleich Therapiestart ergibt einen einzelnen Zeitpunkt.</t>
+  </si>
+  <si>
+    <t>Einzeldosis: Wirkstoffmenge pro Gabe.</t>
+  </si>
+  <si>
+    <t>Einheit: Einheit der Einzeldosis.</t>
+  </si>
+  <si>
+    <t>Anzahl Dosen pro Tag: Häufigkeit der Gabe bzw. geplanten Gabe pro Tag.</t>
+  </si>
+  <si>
+    <t>Beispiel: pro Fall eine Verordnung und eine Gabe.</t>
+  </si>
+  <si>
+    <t>Patient-ID muss in Person vorkommen; leere Patient-ID übernimmt die Patient-ID der vorherigen Zeile.</t>
+  </si>
+  <si>
+    <t>Zeilen ohne gültige Patient-ID werden ignoriert.</t>
+  </si>
+  <si>
+    <t>Fall-Nr ist optional und verweist auf den Encounter aus Fall.</t>
+  </si>
+  <si>
+    <t>Wenn Fall-Nr gefüllt ist, wird Observation.encounter gesetzt.</t>
+  </si>
+  <si>
+    <t>Wenn Fall-Nr leer ist, wird keine Encounter-Referenz gesetzt.</t>
+  </si>
+  <si>
+    <t>Ohne Fall-Nr kann eine spätere Zuordnung nur über Patient-ID und Zeitstempel erfolgen.</t>
+  </si>
+  <si>
+    <t>Bezeichner: Freitext oder Standardwert aus der Auswahlliste.</t>
+  </si>
+  <si>
+    <t>LOINC: Code der klinischen Messung.</t>
+  </si>
+  <si>
+    <t>Wert: numerischer Wert der Messung.</t>
+  </si>
+  <si>
+    <t>Einheit: Einheit der Messung.</t>
+  </si>
+  <si>
+    <t>Zeitstempel: Zeitpunkt der Messung, bevorzugt TT.MM.JJJJ HH:MM:SS.</t>
+  </si>
+  <si>
+    <t>Beispieldaten für Patient 1, Fall 1.</t>
+  </si>
+  <si>
+    <t>Patient-ID muss in Person vorkommen; leere Patient-ID übernimmt die Patient-ID der vorherigen Zeile.</t>
+  </si>
+  <si>
+    <t>Zeilen ohne gültige Patient-ID werden ignoriert.</t>
+  </si>
+  <si>
+    <t>Fall-Nr ist optional und verweist auf Encounter aus Fall.</t>
+  </si>
+  <si>
+    <t>Hier können mehrere Fall-Nummern kommasepariert angegeben werden, z. B. 1,2.</t>
+  </si>
+  <si>
+    <t>Wenn mindestens eine Fall-Nr gefüllt ist, wird DocumentReference.context.encounter gesetzt.</t>
+  </si>
+  <si>
+    <t>Wenn keine Fall-Nr angegeben ist, wird keine Encounter-Referenz gesetzt.</t>
+  </si>
+  <si>
+    <t>Dieses Tabellenblatt hat keinen fachlichen Zeitstempel; DocumentReference.date wird beim Generieren gesetzt.</t>
+  </si>
+  <si>
+    <t>Dateipfad: absoluter Pfad oder relativer Pfad zum Arbeitsverzeichnis des Generators.</t>
+  </si>
+  <si>
+    <t>Embed: ja bettet den Dateiinhalt base64-codiert ein; nein setzt nur die URL.</t>
+  </si>
+  <si>
+    <t>Zeilen, bei denen nur Patient-ID und/oder Fall-Nr gefüllt sind, werden ignoriert.</t>
+  </si>
+  <si>
+    <t>Beispiel: verschiedene Kombinationen aus Fall-Nr, Dateipfad und Embed.</t>
+  </si>
+  <si>
+    <t>Beim unteren Patienten ist ein absoluter Pfad angegeben; bei den anderen ein relativer oder keiner.</t>
   </si>
 </sst>
 </file>
@@ -4254,7 +4593,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -4356,7 +4695,7 @@
         <v>19</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>20</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4387,7 +4726,7 @@
       <c r="L3" s="8"/>
       <c r="M3" s="8"/>
       <c r="N3" s="3" t="s">
-        <v>27</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4418,7 +4757,7 @@
       <c r="L4" s="8"/>
       <c r="M4" s="8"/>
       <c r="N4" s="3" t="s">
-        <v>34</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4477,7 +4816,7 @@
       <c r="L6" s="8"/>
       <c r="M6" s="8"/>
       <c r="N6" s="3" t="s">
-        <v>43</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4508,7 +4847,7 @@
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
       <c r="N7" s="3" t="s">
-        <v>48</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4539,7 +4878,7 @@
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="3" t="s">
-        <v>53</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4570,7 +4909,7 @@
       <c r="L9" s="8"/>
       <c r="M9" s="8"/>
       <c r="N9" s="3" t="s">
-        <v>58</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4629,7 +4968,7 @@
       <c r="L11" s="8"/>
       <c r="M11" s="8"/>
       <c r="N11" s="3" t="s">
-        <v>67</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4639,7 +4978,7 @@
       <c r="L12" s="8"/>
       <c r="M12" s="8"/>
       <c r="N12" s="3" t="s">
-        <v>68</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4649,7 +4988,7 @@
       <c r="L13" s="8"/>
       <c r="M13" s="8"/>
       <c r="N13" s="3" t="s">
-        <v>69</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4659,7 +4998,7 @@
       <c r="L14" s="8"/>
       <c r="M14" s="8"/>
       <c r="N14" s="3" t="s">
-        <v>70</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4669,7 +5008,7 @@
       <c r="L15" s="8"/>
       <c r="M15" s="8"/>
       <c r="N15" s="3" t="s">
-        <v>71</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4679,7 +5018,7 @@
       <c r="L16" s="8"/>
       <c r="M16" s="8"/>
       <c r="N16" s="3" t="s">
-        <v>72</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4696,7 +5035,7 @@
       <c r="L18" s="8"/>
       <c r="M18" s="8"/>
       <c r="N18" s="3" t="s">
-        <v>73</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4706,7 +5045,7 @@
       <c r="L19" s="8"/>
       <c r="M19" s="8"/>
       <c r="N19" s="3" t="s">
-        <v>74</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4716,7 +5055,7 @@
       <c r="L20" s="8"/>
       <c r="M20" s="8"/>
       <c r="N20" s="3" t="s">
-        <v>75</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4726,7 +5065,7 @@
       <c r="L21" s="8"/>
       <c r="M21" s="8"/>
       <c r="N21" s="3" t="s">
-        <v>76</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4736,7 +5075,7 @@
       <c r="L22" s="8"/>
       <c r="M22" s="8"/>
       <c r="N22" s="3" t="s">
-        <v>77</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4746,7 +5085,7 @@
       <c r="L23" s="8"/>
       <c r="M23" s="8"/>
       <c r="N23" s="3" t="s">
-        <v>78</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4756,7 +5095,7 @@
       <c r="L24" s="8"/>
       <c r="M24" s="8"/>
       <c r="N24" s="3" t="s">
-        <v>79</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4773,7 +5112,7 @@
       <c r="L26" s="8"/>
       <c r="M26" s="8"/>
       <c r="N26" s="9" t="s">
-        <v>80</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4797,7 +5136,7 @@
       <c r="L29" s="8"/>
       <c r="M29" s="8"/>
       <c r="N29" s="3" t="s">
-        <v>81</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8861,7 +9200,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -8941,7 +9280,7 @@
         <v>96</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>97</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8962,7 +9301,7 @@
         <v>96</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>99</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8985,7 +9324,7 @@
         <v>102</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>103</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9011,7 +9350,7 @@
         <v>102</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>104</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9043,7 +9382,7 @@
         <v>96</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>105</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9087,7 +9426,7 @@
         <v>101</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>106</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9131,7 +9470,7 @@
         <v>101</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>107</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9174,7 +9513,7 @@
         <v>101</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>13</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9197,7 +9536,7 @@
         <v>93</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>108</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9220,7 +9559,7 @@
         <v>101</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>109</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9264,7 +9603,7 @@
         <v>101</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>110</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9287,7 +9626,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>111</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9310,7 +9649,7 @@
         <v>101</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>112</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9354,7 +9693,7 @@
         <v>101</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>113</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9377,7 +9716,7 @@
         <v>93</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>114</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9400,7 +9739,7 @@
         <v>101</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>115</v>
+        <v>1167</v>
       </c>
     </row>
   </sheetData>
@@ -9437,7 +9776,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -9503,7 +9842,7 @@
         <v>43547</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>97</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9529,7 +9868,7 @@
         <v>43548</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>99</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9555,7 +9894,7 @@
         <v>43549</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>124</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9581,7 +9920,7 @@
         <v>43550</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9607,7 +9946,7 @@
         <v>43551</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>126</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9657,7 +9996,7 @@
         <v>43553</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>127</v>
+        <v>1173</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>128</v>
@@ -9686,7 +10025,7 @@
         <v>43554</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>132</v>
+        <v>1174</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>133</v>
@@ -9715,7 +10054,7 @@
         <v>43555</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>134</v>
+        <v>1175</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>135</v>
@@ -9744,7 +10083,7 @@
         <v>43556</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>136</v>
+        <v>1176</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>137</v>
@@ -9773,7 +10112,7 @@
         <v>43557</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>138</v>
+        <v>1177</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>139</v>
@@ -9871,7 +10210,7 @@
         <v>43561</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>149</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13016,7 +13355,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -13080,7 +13419,7 @@
         <v>174</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>97</v>
+        <v>1179</v>
       </c>
       <c r="H2" s="26"/>
       <c r="J2" s="16"/>
@@ -13105,7 +13444,7 @@
         <v>177</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>178</v>
+        <v>1180</v>
       </c>
       <c r="H3" s="26"/>
       <c r="J3" s="16"/>
@@ -13130,7 +13469,7 @@
         <v>174</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>99</v>
+        <v>1181</v>
       </c>
       <c r="J4" s="16"/>
     </row>
@@ -13154,7 +13493,7 @@
         <v>174</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>124</v>
+        <v>1182</v>
       </c>
       <c r="J5" s="16"/>
     </row>
@@ -13178,7 +13517,7 @@
         <v>177</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>125</v>
+        <v>1183</v>
       </c>
       <c r="J6" s="16"/>
     </row>
@@ -13202,7 +13541,7 @@
         <v>174</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>183</v>
+        <v>1184</v>
       </c>
       <c r="J7" s="16"/>
     </row>
@@ -13249,7 +13588,7 @@
         <v>177</v>
       </c>
       <c r="G9" s="25" t="s">
-        <v>186</v>
+        <v>1185</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="16"/>
@@ -13274,7 +13613,7 @@
         <v>174</v>
       </c>
       <c r="G10" s="25" t="s">
-        <v>187</v>
+        <v>1186</v>
       </c>
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
@@ -13300,7 +13639,7 @@
         <v>174</v>
       </c>
       <c r="G11" s="25" t="s">
-        <v>189</v>
+        <v>1187</v>
       </c>
       <c r="H11" s="16"/>
       <c r="I11" s="16"/>
@@ -13326,7 +13665,7 @@
         <v>177</v>
       </c>
       <c r="G12" s="25" t="s">
-        <v>191</v>
+        <v>1188</v>
       </c>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
@@ -13376,7 +13715,7 @@
         <v>174</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>193</v>
+        <v>1189</v>
       </c>
       <c r="I14" s="16"/>
       <c r="J14" s="16"/>
@@ -14200,7 +14539,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -14256,7 +14595,7 @@
         <v>43547</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>97</v>
+        <v>1190</v>
       </c>
       <c r="H2" s="26"/>
     </row>
@@ -14277,7 +14616,7 @@
         <v>43548</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>178</v>
+        <v>1191</v>
       </c>
       <c r="H3" s="26"/>
     </row>
@@ -14298,7 +14637,7 @@
         <v>43549</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>99</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14318,7 +14657,7 @@
         <v>43550</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>124</v>
+        <v>1193</v>
       </c>
       <c r="H5" s="26"/>
     </row>
@@ -14339,7 +14678,7 @@
         <v>43551</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>125</v>
+        <v>1194</v>
       </c>
       <c r="H6" s="26"/>
     </row>
@@ -14360,7 +14699,7 @@
         <v>43552</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>183</v>
+        <v>1195</v>
       </c>
       <c r="H7" s="26"/>
     </row>
@@ -14400,7 +14739,7 @@
         <v>43554</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>221</v>
+        <v>1196</v>
       </c>
       <c r="H9" s="26"/>
     </row>
@@ -14421,7 +14760,7 @@
         <v>43555</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>224</v>
+        <v>1197</v>
       </c>
       <c r="H10" s="26"/>
     </row>
@@ -14442,7 +14781,7 @@
         <v>43556</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>189</v>
+        <v>1198</v>
       </c>
       <c r="H11" s="26"/>
     </row>
@@ -14500,7 +14839,7 @@
         <v>43559</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>233</v>
+        <v>1199</v>
       </c>
       <c r="H14" s="26"/>
     </row>
@@ -14975,7 +15314,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -15100,7 +15439,7 @@
         <v>1</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>97</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="3" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15150,7 +15489,7 @@
         <v>1</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>178</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="4" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15198,7 +15537,7 @@
         <v>1</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>99</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="5" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15248,7 +15587,7 @@
         <v>1</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>124</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="6" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15296,7 +15635,7 @@
         <v>1</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>125</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="7" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15346,7 +15685,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>183</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="8" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15442,7 +15781,7 @@
         <v>1</v>
       </c>
       <c r="Q9" s="25" t="s">
-        <v>275</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="10" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15490,7 +15829,7 @@
         <v>1</v>
       </c>
       <c r="Q10" s="25" t="s">
-        <v>277</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="11" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15540,7 +15879,7 @@
         <v>1</v>
       </c>
       <c r="Q11" s="25" t="s">
-        <v>279</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="12" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15588,7 +15927,7 @@
         <v>1</v>
       </c>
       <c r="Q12" s="25" t="s">
-        <v>280</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="13" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15638,7 +15977,7 @@
         <v>1</v>
       </c>
       <c r="Q13" s="25" t="s">
-        <v>281</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="14" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15686,7 +16025,7 @@
         <v>1</v>
       </c>
       <c r="Q14" s="25" t="s">
-        <v>282</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="15" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15736,7 +16075,7 @@
         <v>1</v>
       </c>
       <c r="Q15" s="25" t="s">
-        <v>283</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="16" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15784,7 +16123,7 @@
         <v>1</v>
       </c>
       <c r="Q16" s="25" t="s">
-        <v>284</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="17" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15834,7 +16173,7 @@
         <v>1</v>
       </c>
       <c r="Q17" s="25" t="s">
-        <v>285</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="18" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15882,7 +16221,7 @@
         <v>1</v>
       </c>
       <c r="Q18" s="25" t="s">
-        <v>286</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="19" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15932,7 +16271,7 @@
         <v>1</v>
       </c>
       <c r="Q19" s="25" t="s">
-        <v>287</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="20" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15980,7 +16319,7 @@
         <v>1</v>
       </c>
       <c r="Q20" s="25" t="s">
-        <v>288</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="21" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16030,7 +16369,7 @@
         <v>1</v>
       </c>
       <c r="Q21" s="25" t="s">
-        <v>289</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="22" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16078,7 +16417,7 @@
         <v>1</v>
       </c>
       <c r="Q22" s="25" t="s">
-        <v>290</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="23" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16171,7 +16510,7 @@
         <v>1</v>
       </c>
       <c r="Q24" s="9" t="s">
-        <v>291</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17314,7 +17653,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -17380,7 +17719,7 @@
         <v>43546</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>97</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17407,7 +17746,7 @@
         <v>43547</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>178</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17434,7 +17773,7 @@
         <v>43548</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>99</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17461,7 +17800,7 @@
         <v>43549</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>124</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17487,7 +17826,7 @@
         <v>43546</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>125</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17513,7 +17852,7 @@
         <v>43546</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>183</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17564,7 +17903,7 @@
         <v>43547</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>305</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17591,7 +17930,7 @@
         <v>43548</v>
       </c>
       <c r="H10" s="25" t="s">
-        <v>306</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17618,7 +17957,7 @@
         <v>43549</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>307</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17645,7 +17984,7 @@
         <v>43550</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>308</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17671,7 +18010,7 @@
         <v>43546</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>312</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17796,7 +18135,7 @@
         <v>43546</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>316</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18088,7 +18427,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -18128,7 +18467,7 @@
         <v>19</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>97</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18142,7 +18481,7 @@
         <v>322</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>178</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18168,7 +18507,7 @@
         <v>19</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>99</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18185,7 +18524,7 @@
         <v>322</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>323</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18214,7 +18553,7 @@
         <v>19</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>324</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18231,7 +18570,7 @@
         <v>322</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>325</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18254,7 +18593,7 @@
         <v>19</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>183</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18277,7 +18616,7 @@
         <v>19</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>326</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18291,7 +18630,7 @@
         <v>322</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>327</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18305,7 +18644,7 @@
         <v>19</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>328</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18331,12 +18670,12 @@
         <v>329</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>330</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E18" s="9" t="s">
-        <v>331</v>
+        <v>1244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>